<commit_message>
add only bolts and fix inserts assessment
</commit_message>
<xml_diff>
--- a/tests/runners/bolts/config/Flange1.xlsx
+++ b/tests/runners/bolts/config/Flange1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\tests\runners\bolts\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\laghida\Documents\Github\cassy\tests\runners\bolts\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3432AB52-13CB-43EC-8D8F-5F85BB0696C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5138308B-875D-4C6B-8DFC-755720BB3D01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="21600" windowHeight="11385" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-240" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="REs" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="56">
   <si>
     <t>ID</t>
   </si>
@@ -148,9 +148,6 @@
   </si>
   <si>
     <t>bolt</t>
-  </si>
-  <si>
-    <t>insert</t>
   </si>
   <si>
     <t>M12</t>
@@ -702,12 +699,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="11" width="13.7109375" customWidth="1"/>
+    <col min="2" max="11" width="13.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="9" t="s">
         <v>38</v>
       </c>
@@ -742,7 +739,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A2" s="11">
         <v>1</v>
       </c>
@@ -765,10 +762,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I2" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J2" s="14" t="s">
         <v>14</v>
@@ -777,7 +774,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A3" s="16">
         <v>1</v>
       </c>
@@ -800,10 +797,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I3" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J3" s="4" t="s">
         <v>19</v>
@@ -812,7 +809,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A4" s="16">
         <v>1</v>
       </c>
@@ -835,10 +832,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J4" s="4" t="s">
         <v>23</v>
@@ -847,7 +844,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A5" s="16">
         <v>1</v>
       </c>
@@ -870,10 +867,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J5" s="4" t="s">
         <v>23</v>
@@ -882,7 +879,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A6" s="16">
         <v>1</v>
       </c>
@@ -905,10 +902,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I6" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J6" s="4" t="s">
         <v>30</v>
@@ -917,7 +914,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A7" s="16">
         <v>1</v>
       </c>
@@ -940,10 +937,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J7" s="4" t="s">
         <v>30</v>
@@ -952,7 +949,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A8" s="18">
         <v>1</v>
       </c>
@@ -975,10 +972,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I8" s="22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J8" s="22" t="s">
         <v>14</v>
@@ -987,7 +984,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A9">
         <v>2</v>
       </c>
@@ -1010,10 +1007,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I9" s="12" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J9" s="6" t="s">
         <v>14</v>
@@ -1022,7 +1019,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A10">
         <v>2</v>
       </c>
@@ -1045,10 +1042,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J10" s="4" t="s">
         <v>19</v>
@@ -1057,7 +1054,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A11">
         <v>2</v>
       </c>
@@ -1080,10 +1077,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I11" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J11" s="4" t="s">
         <v>23</v>
@@ -1092,7 +1089,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A12">
         <v>2</v>
       </c>
@@ -1115,10 +1112,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="J12" s="4" t="s">
         <v>23</v>
@@ -1127,7 +1124,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A13">
         <v>2</v>
       </c>
@@ -1150,10 +1147,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I13" s="4" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="J13" s="4" t="s">
         <v>30</v>
@@ -1162,7 +1159,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.4">
       <c r="A14">
         <v>2</v>
       </c>
@@ -1185,10 +1182,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="J14" s="4" t="s">
         <v>30</v>
@@ -1197,7 +1194,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>2</v>
       </c>
@@ -1220,10 +1217,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I15" s="22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J15" s="6" t="s">
         <v>14</v>
@@ -1240,12 +1237,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ED687A43-EC33-423B-A6DD-5E62238FF478}">
   <dimension ref="A1:M5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="13" width="15.7109375" customWidth="1"/>
+    <col min="2" max="13" width="15.69140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="29.6" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A1" s="10" t="s">
         <v>38</v>
       </c>
@@ -1274,10 +1271,10 @@
         <v>37</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>48</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>49</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>8</v>
@@ -1286,7 +1283,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1327,12 +1324,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C3" s="24" t="s">
         <v>11</v>
@@ -1368,7 +1365,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A4">
         <v>2</v>
       </c>
@@ -1409,12 +1406,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A5">
         <v>2</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C5" s="24" t="s">
         <v>11</v>
@@ -1457,34 +1454,34 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE19EBD1-4CCE-4BC0-AB0E-DF85D1968C61}">
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="2" max="2" width="11.85546875" customWidth="1"/>
-    <col min="3" max="3" width="10.28515625" customWidth="1"/>
+    <col min="2" max="2" width="11.84375" customWidth="1"/>
+    <col min="3" max="3" width="10.3046875" customWidth="1"/>
     <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A1" t="s">
         <v>38</v>
       </c>
       <c r="B1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" t="s">
         <v>42</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>43</v>
       </c>
-      <c r="D1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C2" t="s">
         <v>39</v>
@@ -1493,45 +1490,17 @@
         <v>200000</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" s="7">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>2</v>
-      </c>
-      <c r="B4" t="s">
-        <v>41</v>
-      </c>
-      <c r="C4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" s="7">
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C5" t="s">
-        <v>40</v>
-      </c>
-      <c r="D5" s="7">
         <v>200000</v>
       </c>
     </row>
@@ -1543,26 +1512,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{104CCDBF-B7FA-4C2C-914E-1618DEA9FA0D}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="11.85546875" customWidth="1"/>
+    <col min="1" max="1" width="11.84375" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="B1" s="8" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>